<commit_message>
Reorganize data/ by tab first, then estate; rename tabs to match
data/<estate>/ becomes data/Agronomic Assessment/<estate>/, with matching
(currently empty) data/Bunch Development/<estate>/ and data/Yield Map/<estate>/
scaffolded for future real WC2/WC4 data. Updated build_wc1_assessment.py,
setup_folders.py, setup_accounts.py, and app.py's media route to match.

Tabs renamed to follow the folder names: "WC1 Assessment" -> "Agronomic
Assessment", "Yield" -> "Yield Map" (Bunch Development unchanged).

Regenerated outputs/WC1_agronomic_assessment_synced.xlsx so frame_relpath
reflects the new location.
</commit_message>
<xml_diff>
--- a/outputs/WC1_agronomic_assessment_synced.xlsx
+++ b/outputs/WC1_agronomic_assessment_synced.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00144.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00144.jpg</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00161.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00161.jpg</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00162.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00162.jpg</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00179.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00179.jpg</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00185.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00185.jpg</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00188.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00188.jpg</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00195.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00195.jpg</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00230.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00230.jpg</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00248.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00248.jpg</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00264.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00264.jpg</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00269.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00269.jpg</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00282.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00282.jpg</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00292.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00292.jpg</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00299.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00299.jpg</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00313.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00313.jpg</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113101712_0103_D/frame_00397.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113101712_0103_D/frame_00397.jpg</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00001.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00001.jpg</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00017.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00017.jpg</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00030.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00030.jpg</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00097.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00097.jpg</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00130.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00130.jpg</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00214.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00214.jpg</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00247.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00247.jpg</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00264.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00264.jpg</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00278.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00278.jpg</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00300.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00300.jpg</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00324.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00324.jpg</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00362.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00362.jpg</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113102453_0104_D/frame_00371.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113102453_0104_D/frame_00371.jpg</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00092.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00092.jpg</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00161.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00161.jpg</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00248.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00248.jpg</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00285.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00285.jpg</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00287.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00287.jpg</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00360.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00360.jpg</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00379.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00379.jpg</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00395.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00395.jpg</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113103248_0105_D/frame_00405.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113103248_0105_D/frame_00405.jpg</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00012.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00012.jpg</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00018.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00018.jpg</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00039.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00039.jpg</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00042.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00042.jpg</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00084.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00084.jpg</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00115.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00115.jpg</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00137.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00137.jpg</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00176.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00176.jpg</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00237.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00237.jpg</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00267.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00267.jpg</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00313.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00313.jpg</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00338.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00338.jpg</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260113104029_0106_D/frame_00358.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260113104029_0106_D/frame_00358.jpg</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00036.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00036.jpg</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00039.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00039.jpg</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00050.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00050.jpg</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00067.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00067.jpg</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00071.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00071.jpg</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00104.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00104.jpg</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00109.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00109.jpg</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00111.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00111.jpg</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00118.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00118.jpg</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00127.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00127.jpg</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00133.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00133.jpg</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00160.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00160.jpg</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00167.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00167.jpg</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00172.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00172.jpg</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00185.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00185.jpg</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00204.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00204.jpg</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00216.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00216.jpg</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00224.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00224.jpg</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00269.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00269.jpg</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00282.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00282.jpg</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00322.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00322.jpg</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00329.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00329.jpg</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00386.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00386.jpg</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00392.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00392.jpg</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00395.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00395.jpg</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00397.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00397.jpg</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115103221_0001_D/frame_00403.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115103221_0001_D/frame_00403.jpg</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00003.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00003.jpg</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -6607,7 +6607,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00012.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00012.jpg</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00018.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00018.jpg</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -6759,7 +6759,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00059.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00059.jpg</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -6835,7 +6835,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00060.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00060.jpg</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00064.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00064.jpg</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00065.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00065.jpg</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -7063,7 +7063,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00068.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00068.jpg</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -7139,7 +7139,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00084.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00084.jpg</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00085.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00085.jpg</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00086.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00086.jpg</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00111.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00111.jpg</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -7443,7 +7443,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00116.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00116.jpg</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00136.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00136.jpg</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00152.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00152.jpg</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00158.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00158.jpg</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00181.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00181.jpg</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00198.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00198.jpg</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00223.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00223.jpg</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00225.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00225.jpg</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
@@ -8051,7 +8051,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00231.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00231.jpg</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00258.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00258.jpg</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00324.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00324.jpg</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00325.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00325.jpg</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00350.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00350.jpg</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -8431,7 +8431,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104002_0002_D/frame_00377.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104002_0002_D/frame_00377.jpg</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -8507,7 +8507,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00061.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00061.jpg</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr"/>
@@ -8575,7 +8575,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00063.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00063.jpg</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -8643,7 +8643,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00070.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00070.jpg</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00076.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00076.jpg</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr"/>
@@ -8779,7 +8779,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00079.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00079.jpg</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr"/>
@@ -8847,7 +8847,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00085.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00085.jpg</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -8915,7 +8915,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00123.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00123.jpg</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00143.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00143.jpg</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr"/>
@@ -9051,7 +9051,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00146.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00146.jpg</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -9119,7 +9119,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00155.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00155.jpg</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -9187,7 +9187,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00163.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00163.jpg</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -9255,7 +9255,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00168.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00168.jpg</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -9323,7 +9323,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00207.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00207.jpg</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -9391,7 +9391,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00212.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00212.jpg</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -9459,7 +9459,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00227.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00227.jpg</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00230.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00230.jpg</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -9595,7 +9595,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00275.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00275.jpg</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr"/>
@@ -9663,7 +9663,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00288.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00288.jpg</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -9731,7 +9731,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00300.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00300.jpg</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr"/>
@@ -9799,7 +9799,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00302.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00302.jpg</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr"/>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00327.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00327.jpg</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr"/>
@@ -9935,7 +9935,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00365.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00365.jpg</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -10003,7 +10003,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00377.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00377.jpg</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -10071,7 +10071,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00390.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00390.jpg</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -10139,7 +10139,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00404.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00404.jpg</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -10207,7 +10207,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00407.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00407.jpg</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00423.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00423.jpg</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -10343,7 +10343,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00445.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00445.jpg</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -10411,7 +10411,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>data/Serdang-2/DJI_20260115104912_0003_D/frame_00460.jpg</t>
+          <t>data/Agronomic Assessment/Serdang-2/DJI_20260115104912_0003_D/frame_00460.jpg</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr"/>

</xml_diff>